<commit_message>
Re-cut projections and package to January-takeout base case (Rev 3.10)
Per the executed MIPA: $31,250/mo Sep-Dec equity-funded, ~$258,489
balloon retired by SBA at the 51% transfer 1/15/2027 (avoids seller
guaranties under partial-CHOW rules); September takeout kept as upside
toggle. QA 24/24. Disclosed finding: the slow-census downside now needs
a ~$375K facility vs the $250K base revolver. UOP workbook, debt
schedule, checklist memo, addendum, assumptions, cover/reply emails,
and Business Plan Rev 6.00 all updated to the January base.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GAHLyfqLR9bxwN2jm6VjPU
</commit_message>
<xml_diff>
--- a/sba_application/13_checklist_response_2026-07-16/UOP Azalea Refuge Rev1.00.xlsx
+++ b/sba_application/13_checklist_response_2026-07-16/UOP Azalea Refuge Rev1.00.xlsx
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F40"/>
+  <dimension ref="A1:F42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -504,7 +504,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">   of which: seller-financed balance at 6% (SBA takeout Sept 2026)</t>
+          <t xml:space="preserve">   of which: seller-financed balance at 6% (SBA takeout at the 51% transfer, 1/15/2027)</t>
         </is>
       </c>
       <c r="B7" s="4">
@@ -652,7 +652,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>SBA 7(a) loan (retires seller balance Sept 2026 + working capital)</t>
+          <t>SBA 7(a) loan (funds Jan 2027: seller balloon takeout + working capital)</t>
         </is>
       </c>
       <c r="B20" s="4" t="n">
@@ -727,7 +727,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Loan amount</t>
+          <t>Loan amount (funds ~1/15/2027, concurrent with the 51% transfer)</t>
         </is>
       </c>
       <c r="B27" s="4">
@@ -863,14 +863,28 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Note: the Rev 3.00 proforma conservatively models debt service at a 36-month</t>
+          <t>BASE CASE: SBA funds January 2027 at the 51% transfer (a clean 100% change of ownership;</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>amortization ($15,211/mo). Actual 7(a) terms above cut that by more than half.</t>
+          <t>no seller guaranties required). September funding is an UPSIDE if a lender can paper the</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>partial-CHOW guaranty rules. The Rev 3.10 proforma conservatively models the takeout at a</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>36-month amortization ($7,957/mo from Feb); actual 7(a) terms above are the cheaper case.</t>
         </is>
       </c>
     </row>
@@ -921,7 +935,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Purpose: fund operations through the Medicare payment lag (NOE-to-cash ~30-60 days) while census ramps to break-even (~17-18 patients, crossed month 2-3 per the Rev 3.00 proforma).</t>
+          <t>Purpose: fund operations through the Medicare payment lag (NOE-to-cash ~30-60 days) while census ramps to break-even (~17-18 patients, crossed month 2-3 per the Rev 3.10 proforma). BASE CASE: the SBA loan funds ~1/15/2027; amounts shown before then are bridged on an interim LOC (peak need ~$183K base / ~$375K downside) and repaid from the reserve at SBA funding.</t>
         </is>
       </c>
     </row>
@@ -1512,7 +1526,7 @@
     <row r="19">
       <c r="A19" s="10" t="inlineStr">
         <is>
-          <t>gross monthly operating costs and collections are in the attached Rev 3.00 proforma (36 monthly periods).</t>
+          <t>gross monthly operating costs and collections are in the attached Rev 3.10 proforma (36 monthly periods).</t>
         </is>
       </c>
     </row>
@@ -1526,14 +1540,21 @@
     <row r="21">
       <c r="A21" s="10" t="inlineStr">
         <is>
-          <t>Prior structure carried a $672,000 reserve; the current structure needs $235,000 because the acquisition is</t>
+          <t>Prior structure carried a $672,000 reserve; the current structure needs $235,000 because the license is</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="10" t="inlineStr">
         <is>
-          <t>seller-financed to September (SBA takeout), the license is billing-ready day one, and equity covers the down payment.</t>
+          <t>billing-ready day one and equity covers the down payment plus the seller installments through December.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="10" t="inlineStr">
+        <is>
+          <t>Base case peak interim-LOC need before SBA funding is ~$183K; the documented slow-census downside needs a</t>
         </is>
       </c>
     </row>
@@ -1559,7 +1580,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1638,97 +1659,159 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>SBA 7(a) funds - full note takeout (principal)</t>
+          <t>Monthly installment ($31,250 incl. 6% interest)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Sept 2026</t>
-        </is>
-      </c>
-      <c r="C6" s="4">
-        <f>D5</f>
-        <v/>
-      </c>
-      <c r="D6" s="4">
-        <f>D5-C6</f>
-        <v/>
+          <t>9/1/2026</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>31250</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>SBA loan proceeds</t>
+          <t>Equity injection</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Accrued interest at takeout (est. 1 month at 6%)</t>
+          <t>Monthly installment</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Sept 2026</t>
-        </is>
-      </c>
-      <c r="C7" s="4">
-        <f>ROUND(D5*0.06/12,0)</f>
-        <v/>
-      </c>
-      <c r="D7" s="4" t="n">
-        <v>0</v>
+          <t>10/1/2026</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>31250</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>SBA loan proceeds</t>
+          <t>Equity injection</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Monthly installment</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>11/1/2026</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>31250</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Equity injection</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Remaining 51% of membership interests transfer 1/15/2027 - the first date past 36 months from the</t>
+          <t>Monthly installment</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>12/1/2026</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="n">
+        <v>31250</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Equity injection</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>company's CMS certification effective date (1/8/2024), as required by 42 CFR 424.550(b).</t>
+          <t>Final payment per MIPA amortization (Exhibit C)</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>1/15/2027</t>
+        </is>
+      </c>
+      <c r="C10" s="11" t="n">
+        <v>258489.46</v>
+      </c>
+      <c r="D10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>SBA 7(a) proceeds</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>If SBA funding is later than September (contract fallback per MIPA):</t>
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>BASE CASE: the SBA 7(a) loan funds ~1/15/2027, concurrent with the transfer of the remaining 51%</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Monthly installment (from 9/1/2026)</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="n">
-        <v>31250</v>
+          <t>of membership interests - the first date past 36 months from the company's CMS certification</t>
+        </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Final payment 1/15/2027 (per MIPA amortization)</t>
-        </is>
-      </c>
-      <c r="B14" s="11" t="n">
-        <v>258489.46</v>
+          <t>effective date (1/8/2024) per 42 CFR 424.550(b). Funding at the 100% transfer avoids the seller-</t>
+        </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>The note is prepayable at any time without penalty, so SBA takeout can occur any month.</t>
+          <t>guaranty requirements that apply to SBA loans made during a partial change of ownership.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>UPSIDE - September takeout (note is prepayable without penalty):</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>If a lender can fund September 2026, payoff is $375,000 + ~$1,875 accrued interest, saving four</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>installments and ~$8,500 of seller interest. Requires the lender to paper seller guaranties under</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>the partial-change-of-ownership rules, so it is presented as upside, not base.</t>
         </is>
       </c>
     </row>

</xml_diff>